<commit_message>
update in management files
No arquivo '0FUMO - Planejamento e Controle do Projeto.xlsx' foi atualizado o planejamento de entregas, atualizando os dois novos casos de uso implementados, UC Registrar Eventos e UC Realizar Avaliacao Inicial.

No arquivo '0FUMO - Checklist Verificacao de Projeto.xlsx' foi preenchido o checklist da fase de Construcao.
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/0FUMO - Checklist Verificacao de Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/0FUMO - Checklist Verificacao de Projeto.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\E303327\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Downloads\Git subir\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA0F8B3-4EAB-40A5-BDFB-3687109EAA68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA18C592-C362-460C-9EBE-69F19692E19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicadores" sheetId="1" r:id="rId1"/>
@@ -389,7 +389,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="120">
   <si>
     <t>IAP - Indicador de Aderência ao Processo (70% a 100%)</t>
   </si>
@@ -1206,15 +1206,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -1224,6 +1221,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1231,16 +1229,18 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1263,7 +1263,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -1279,7 +1279,7 @@
           <c:order val="0"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:srgbClr val="5B9BD5"/>
             </a:solidFill>
             <a:ln cmpd="sng">
               <a:solidFill>
@@ -1335,7 +1335,7 @@
                   <c:v>0.85</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1506,7 +1506,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -1553,7 +1553,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:srgbClr val="5B9BD5"/>
             </a:solidFill>
             <a:ln cmpd="sng">
               <a:solidFill>
@@ -1673,7 +1673,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent2"/>
+              <a:srgbClr val="ED7D31"/>
             </a:solidFill>
             <a:ln cmpd="sng">
               <a:solidFill>
@@ -1793,7 +1793,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent3"/>
+              <a:srgbClr val="A5A5A5"/>
             </a:solidFill>
             <a:ln cmpd="sng">
               <a:solidFill>
@@ -1913,7 +1913,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent4"/>
+              <a:srgbClr val="FFC000"/>
             </a:solidFill>
             <a:ln cmpd="sng">
               <a:solidFill>
@@ -2187,7 +2187,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -2762,7 +2762,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -2870,10 +2870,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -2888,19 +2888,19 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.8</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.8</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2983,7 +2983,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3108,7 +3108,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -3197,22 +3197,22 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -3221,16 +3221,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3361,7 +3361,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-BR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -4353,10 +4353,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
+      <c r="B1" s="38"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -4388,9 +4388,9 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="e">
+      <c r="B5" s="3">
         <f>'Ver-Construção1'!$F$2</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -7903,42 +7903,42 @@
       <c r="A23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="6" t="e">
+      <c r="B23" s="6">
         <f>('Ver-Construção1'!$G$6/SUM('Ver-Construção1'!$G$6:'Ver-Construção1'!$J$6))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C23" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="C23" s="7">
         <f>('Ver-Construção1'!$H$6/SUM('Ver-Construção1'!$G$6:'Ver-Construção1'!$J$6))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D23" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="D23" s="7">
         <f>('Ver-Construção1'!$I$6/SUM('Ver-Construção1'!$G$6:'Ver-Construção1'!$J$6))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E23" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="E23" s="7">
         <f>('Ver-Construção1'!$J$6/SUM('Ver-Construção1'!$G$6:'Ver-Construção1'!$J$6))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B24" s="6" t="e">
+      <c r="B24" s="6">
         <f>('Ver-Construção1'!$G$8/SUM('Ver-Construção1'!$G$8:'Ver-Construção1'!$J$8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C24" s="7" t="e">
+        <v>1</v>
+      </c>
+      <c r="C24" s="7">
         <f>('Ver-Construção1'!$H$8/SUM('Ver-Construção1'!$G$8:'Ver-Construção1'!$J$8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D24" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="D24" s="7">
         <f>('Ver-Construção1'!$I$8/SUM('Ver-Construção1'!$G$8:'Ver-Construção1'!$J$8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E24" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="E24" s="7">
         <f>('Ver-Construção1'!$J$8/SUM('Ver-Construção1'!$G$8:'Ver-Construção1'!$J$8))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="M24" s="5" t="s">
         <v>7</v>
@@ -7960,21 +7960,21 @@
       <c r="A25" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="6" t="e">
+      <c r="B25" s="6">
         <f>('Ver-Construção1'!$G$10/SUM('Ver-Construção1'!$G$10:'Ver-Construção1'!$J$10))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C25" s="7" t="e">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C25" s="7">
         <f>('Ver-Construção1'!$G$10/SUM('Ver-Construção1'!$G$10:'Ver-Construção1'!$J$10))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D25" s="7" t="e">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D25" s="7">
         <f>('Ver-Construção1'!$I$10/SUM('Ver-Construção1'!$G$10:'Ver-Construção1'!$J$10))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E25" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="E25" s="7">
         <f>('Ver-Construção1'!$J$10/SUM('Ver-Construção1'!$G$10:'Ver-Construção1'!$J$10))</f>
-        <v>#DIV/0!</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="M25" s="5" t="s">
         <v>13</v>
@@ -8000,21 +8000,21 @@
       <c r="A26" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="7" t="e">
+      <c r="B26" s="7">
         <f>('Ver-Construção1'!$G$14/SUM('Ver-Construção1'!$G$14:'Ver-Construção1'!$J$14))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C26" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="C26" s="7">
         <f>('Ver-Construção1'!$H$14/SUM('Ver-Construção1'!$G$14:'Ver-Construção1'!$J$14))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D26" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="D26" s="7">
         <f>('Ver-Construção1'!$I$14/SUM('Ver-Construção1'!$G$14:'Ver-Construção1'!$J$14))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E26" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="E26" s="7">
         <f>('Ver-Construção1'!$J$14/SUM('Ver-Construção1'!$G$14:'Ver-Construção1'!$J$14))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="M26" s="5" t="s">
         <v>14</v>
@@ -8080,21 +8080,21 @@
       <c r="A28" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="7" t="e">
+      <c r="B28" s="7">
         <f>('Ver-Construção1'!$G$16/SUM('Ver-Construção1'!$G$16:'Ver-Construção1'!$J$16))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C28" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="C28" s="7">
         <f>('Ver-Construção1'!$H$16/SUM('Ver-Construção1'!$G$16:'Ver-Construção1'!$J$16))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D28" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="D28" s="7">
         <f>('Ver-Construção1'!$I$16/SUM('Ver-Construção1'!$G$16:'Ver-Construção1'!$J$16))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E28" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="E28" s="7">
         <f>('Ver-Construção1'!$J$16/SUM('Ver-Construção1'!$G$16:'Ver-Construção1'!$J$16))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="M28" s="5" t="s">
         <v>16</v>
@@ -8160,21 +8160,21 @@
       <c r="A30" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B30" s="7" t="e">
+      <c r="B30" s="7">
         <f>('Ver-Construção1'!$G$18/SUM('Ver-Construção1'!$G$18:'Ver-Construção1'!$J$18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C30" s="7" t="e">
+        <v>0.8</v>
+      </c>
+      <c r="C30" s="7">
         <f>('Ver-Construção1'!$H$18/SUM('Ver-Construção1'!$G$18:'Ver-Construção1'!$J$18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D30" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="D30" s="7">
         <f>('Ver-Construção1'!$I$18/SUM('Ver-Construção1'!$G$18:'Ver-Construção1'!$J$18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E30" s="7" t="e">
+        <v>0.2</v>
+      </c>
+      <c r="E30" s="7">
         <f>('Ver-Construção1'!$J$18/SUM('Ver-Construção1'!$G$18:'Ver-Construção1'!$J$18))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="M30" s="5" t="s">
         <v>18</v>
@@ -8200,21 +8200,21 @@
       <c r="A31" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B31" s="7" t="e">
+      <c r="B31" s="7">
         <f>('Ver-Construção1'!$G$24/SUM('Ver-Construção1'!$G$24:'Ver-Construção1'!$J$24))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C31" s="7" t="e">
+        <v>0.8</v>
+      </c>
+      <c r="C31" s="7">
         <f>('Ver-Construção1'!$H$24/SUM('Ver-Construção1'!$G$24:'Ver-Construção1'!$J$24))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D31" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="D31" s="7">
         <f>('Ver-Construção1'!$I$24/SUM('Ver-Construção1'!$G$24:'Ver-Construção1'!$J$24))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E31" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="E31" s="7">
         <f>('Ver-Construção1'!$J$24/SUM('Ver-Construção1'!$G$24:'Ver-Construção1'!$J$24))</f>
-        <v>#DIV/0!</v>
+        <v>0.2</v>
       </c>
       <c r="M31" s="5" t="s">
         <v>22</v>
@@ -8240,21 +8240,21 @@
       <c r="A32" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="7" t="e">
+      <c r="B32" s="7">
         <f>('Ver-Construção1'!$G$30/SUM('Ver-Construção1'!$G$30:'Ver-Construção1'!$J$30))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C32" s="7" t="e">
+        <v>0.4</v>
+      </c>
+      <c r="C32" s="7">
         <f>('Ver-Construção1'!$H$30/SUM('Ver-Construção1'!$G$30:'Ver-Construção1'!$J$30))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D32" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="D32" s="7">
         <f>('Ver-Construção1'!$I$30/SUM('Ver-Construção1'!$G$30:'Ver-Construção1'!$J$30))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E32" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="E32" s="7">
         <f>('Ver-Construção1'!$J$30/SUM('Ver-Construção1'!$G$30:'Ver-Construção1'!$J$30))</f>
-        <v>#DIV/0!</v>
+        <v>0.6</v>
       </c>
       <c r="M32" s="5" t="s">
         <v>26</v>
@@ -8280,21 +8280,21 @@
       <c r="A33" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B33" s="7" t="e">
+      <c r="B33" s="7">
         <f>('Ver-Construção1'!$G$36/SUM('Ver-Construção1'!$G$36:'Ver-Construção1'!$J$36))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C33" s="7" t="e">
+        <v>1</v>
+      </c>
+      <c r="C33" s="7">
         <f>('Ver-Construção1'!$H$36/SUM('Ver-Construção1'!$G$36:'Ver-Construção1'!$J$36))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D33" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="D33" s="7">
         <f>('Ver-Construção1'!$I$36/SUM('Ver-Construção1'!$G$36:'Ver-Construção1'!$J$36))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E33" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="E33" s="7">
         <f>('Ver-Construção1'!$J$36/SUM('Ver-Construção1'!$G$36:'Ver-Construção1'!$J$36))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="M33" s="5" t="s">
         <v>27</v>
@@ -8320,21 +8320,21 @@
       <c r="A34" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B34" s="7" t="e">
+      <c r="B34" s="7">
         <f>('Ver-Construção1'!$G$41/SUM('Ver-Construção1'!$G$41:'Ver-Construção1'!$J$41))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C34" s="7" t="e">
+        <v>0.5</v>
+      </c>
+      <c r="C34" s="7">
         <f>('Ver-Construção1'!$H$41/SUM('Ver-Construção1'!$G$41:'Ver-Construção1'!$J$41))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D34" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="D34" s="7">
         <f>('Ver-Construção1'!$I$41/SUM('Ver-Construção1'!$G$41:'Ver-Construção1'!$J$41))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E34" s="7" t="e">
+        <v>0</v>
+      </c>
+      <c r="E34" s="7">
         <f>('Ver-Construção1'!$J$41/SUM('Ver-Construção1'!$G$41:'Ver-Construção1'!$J$41))</f>
-        <v>#DIV/0!</v>
+        <v>0.5</v>
       </c>
       <c r="M34" s="5" t="s">
         <v>28</v>
@@ -9408,20 +9408,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
     </row>
     <row r="2" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="30"/>
+      <c r="B2" s="38"/>
       <c r="C2" s="8">
         <v>46113</v>
       </c>
@@ -9438,11 +9438,11 @@
       <c r="A3" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="30"/>
+      <c r="B3" s="38"/>
       <c r="C3" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="47" t="s">
         <v>34</v>
       </c>
       <c r="E3" s="43"/>
@@ -9469,7 +9469,7 @@
       </c>
     </row>
     <row r="5" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="29" t="s">
         <v>41</v>
       </c>
       <c r="B5" s="15"/>
@@ -9497,7 +9497,7 @@
       </c>
     </row>
     <row r="6" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="46"/>
+      <c r="A6" s="32"/>
       <c r="B6" s="18">
         <v>1</v>
       </c>
@@ -9511,7 +9511,7 @@
       <c r="F6" s="19"/>
     </row>
     <row r="7" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="29" t="s">
         <v>44</v>
       </c>
       <c r="B7" s="15"/>
@@ -9539,7 +9539,7 @@
       </c>
     </row>
     <row r="8" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="32"/>
+      <c r="A8" s="30"/>
       <c r="B8" s="21">
         <v>2</v>
       </c>
@@ -9553,7 +9553,7 @@
       <c r="F8" s="19"/>
     </row>
     <row r="9" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32"/>
+      <c r="A9" s="30"/>
       <c r="B9" s="18">
         <v>3</v>
       </c>
@@ -9567,7 +9567,7 @@
       <c r="F9" s="19"/>
     </row>
     <row r="10" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="18">
         <v>4</v>
       </c>
@@ -9581,7 +9581,7 @@
       <c r="F10" s="19"/>
     </row>
     <row r="11" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="32"/>
+      <c r="A11" s="30"/>
       <c r="B11" s="18">
         <v>5</v>
       </c>
@@ -9615,7 +9615,7 @@
       <c r="Z11" s="23"/>
     </row>
     <row r="12" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32"/>
+      <c r="A12" s="30"/>
       <c r="B12" s="18">
         <v>6</v>
       </c>
@@ -9629,7 +9629,7 @@
       <c r="F12" s="19"/>
     </row>
     <row r="13" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
+      <c r="A13" s="30"/>
       <c r="B13" s="15"/>
       <c r="C13" s="16" t="s">
         <v>14</v>
@@ -9655,7 +9655,7 @@
       </c>
     </row>
     <row r="14" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="32"/>
+      <c r="A14" s="30"/>
       <c r="B14" s="24">
         <v>7</v>
       </c>
@@ -9669,7 +9669,7 @@
       <c r="F14" s="19"/>
     </row>
     <row r="15" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32"/>
+      <c r="A15" s="30"/>
       <c r="B15" s="18">
         <v>8</v>
       </c>
@@ -9703,7 +9703,7 @@
       <c r="Z15" s="23"/>
     </row>
     <row r="16" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="32"/>
+      <c r="A16" s="30"/>
       <c r="B16" s="18">
         <v>9</v>
       </c>
@@ -9737,7 +9737,7 @@
       <c r="Z16" s="23"/>
     </row>
     <row r="17" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="32"/>
+      <c r="A17" s="30"/>
       <c r="B17" s="24">
         <v>10</v>
       </c>
@@ -9771,7 +9771,7 @@
       <c r="Z17" s="23"/>
     </row>
     <row r="18" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
+      <c r="A18" s="30"/>
       <c r="B18" s="18">
         <v>11</v>
       </c>
@@ -9805,7 +9805,7 @@
       <c r="Z18" s="23"/>
     </row>
     <row r="19" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
+      <c r="A19" s="30"/>
       <c r="B19" s="15"/>
       <c r="C19" s="16" t="s">
         <v>57</v>
@@ -9831,7 +9831,7 @@
       </c>
     </row>
     <row r="20" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
+      <c r="A20" s="30"/>
       <c r="B20" s="24">
         <v>12</v>
       </c>
@@ -9845,7 +9845,7 @@
       <c r="F20" s="19"/>
     </row>
     <row r="21" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="32"/>
+      <c r="A21" s="30"/>
       <c r="B21" s="18">
         <v>13</v>
       </c>
@@ -9859,7 +9859,7 @@
       <c r="F21" s="19"/>
     </row>
     <row r="22" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="32"/>
+      <c r="A22" s="30"/>
       <c r="B22" s="15"/>
       <c r="C22" s="16" t="s">
         <v>16</v>
@@ -9885,7 +9885,7 @@
       </c>
     </row>
     <row r="23" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32"/>
+      <c r="A23" s="30"/>
       <c r="B23" s="24">
         <v>14</v>
       </c>
@@ -9899,7 +9899,7 @@
       <c r="F23" s="19"/>
     </row>
     <row r="24" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="32"/>
+      <c r="A24" s="30"/>
       <c r="B24" s="18">
         <v>15</v>
       </c>
@@ -9913,7 +9913,7 @@
       <c r="F24" s="19"/>
     </row>
     <row r="25" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="32"/>
+      <c r="A25" s="30"/>
       <c r="B25" s="15"/>
       <c r="C25" s="16" t="s">
         <v>17</v>
@@ -9939,7 +9939,7 @@
       </c>
     </row>
     <row r="26" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="32"/>
+      <c r="A26" s="30"/>
       <c r="B26" s="24">
         <v>16</v>
       </c>
@@ -9953,7 +9953,7 @@
       <c r="F26" s="19"/>
     </row>
     <row r="27" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="33"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="18">
         <v>17</v>
       </c>
@@ -9967,7 +9967,7 @@
       <c r="F27" s="19"/>
     </row>
     <row r="28" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="31"/>
+      <c r="A28" s="46"/>
       <c r="B28" s="15"/>
       <c r="C28" s="16" t="s">
         <v>23</v>
@@ -9993,7 +9993,7 @@
       </c>
     </row>
     <row r="29" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="32"/>
+      <c r="A29" s="30"/>
       <c r="B29" s="24">
         <v>21</v>
       </c>
@@ -10007,7 +10007,7 @@
       <c r="F29" s="19"/>
     </row>
     <row r="30" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="32"/>
+      <c r="A30" s="30"/>
       <c r="B30" s="18">
         <v>22</v>
       </c>
@@ -10021,7 +10021,7 @@
       <c r="F30" s="19"/>
     </row>
     <row r="31" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="32"/>
+      <c r="A31" s="30"/>
       <c r="B31" s="18">
         <v>23</v>
       </c>
@@ -10035,7 +10035,7 @@
       <c r="F31" s="19"/>
     </row>
     <row r="32" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="32"/>
+      <c r="A32" s="30"/>
       <c r="B32" s="18">
         <v>24</v>
       </c>
@@ -10049,7 +10049,7 @@
       <c r="F32" s="19"/>
     </row>
     <row r="33" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32"/>
+      <c r="A33" s="30"/>
       <c r="B33" s="18">
         <v>25</v>
       </c>
@@ -10063,7 +10063,7 @@
       <c r="F33" s="19"/>
     </row>
     <row r="34" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="32"/>
+      <c r="A34" s="30"/>
       <c r="B34" s="18">
         <v>26</v>
       </c>
@@ -10076,7 +10076,7 @@
       <c r="F34" s="19"/>
     </row>
     <row r="35" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="32"/>
+      <c r="A35" s="30"/>
       <c r="B35" s="18">
         <v>27</v>
       </c>
@@ -10090,7 +10090,7 @@
       <c r="F35" s="19"/>
     </row>
     <row r="36" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="33"/>
+      <c r="A36" s="31"/>
       <c r="B36" s="18">
         <v>28</v>
       </c>
@@ -10104,7 +10104,7 @@
       <c r="F36" s="19"/>
     </row>
     <row r="37" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="34" t="s">
+      <c r="A37" s="33" t="s">
         <v>69</v>
       </c>
       <c r="B37" s="15"/>
@@ -10132,7 +10132,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="35"/>
+      <c r="A38" s="34"/>
       <c r="B38" s="24">
         <v>30</v>
       </c>
@@ -10146,7 +10146,7 @@
       <c r="F38" s="19"/>
     </row>
     <row r="39" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="35"/>
+      <c r="A39" s="34"/>
       <c r="B39" s="18">
         <v>31</v>
       </c>
@@ -10160,7 +10160,7 @@
       <c r="F39" s="19"/>
     </row>
     <row r="40" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="35"/>
+      <c r="A40" s="34"/>
       <c r="B40" s="18">
         <v>32</v>
       </c>
@@ -10174,7 +10174,7 @@
       <c r="F40" s="19"/>
     </row>
     <row r="41" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="36"/>
+      <c r="A41" s="35"/>
       <c r="B41" s="18">
         <v>33</v>
       </c>
@@ -14062,20 +14062,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
     </row>
     <row r="2" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="30"/>
+      <c r="B2" s="38"/>
       <c r="C2" s="8">
         <v>46141</v>
       </c>
@@ -14092,11 +14092,11 @@
       <c r="A3" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="30"/>
+      <c r="B3" s="38"/>
       <c r="C3" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="D3" s="47" t="s">
+      <c r="D3" s="42" t="s">
         <v>34</v>
       </c>
       <c r="E3" s="43"/>
@@ -14123,7 +14123,7 @@
       </c>
     </row>
     <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="29" t="s">
         <v>44</v>
       </c>
       <c r="B5" s="15"/>
@@ -14135,7 +14135,7 @@
       <c r="F5" s="17"/>
     </row>
     <row r="6" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="32"/>
+      <c r="A6" s="30"/>
       <c r="B6" s="18">
         <v>1</v>
       </c>
@@ -14165,7 +14165,7 @@
       </c>
     </row>
     <row r="7" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="32"/>
+      <c r="A7" s="30"/>
       <c r="B7" s="15"/>
       <c r="C7" s="16" t="s">
         <v>14</v>
@@ -14175,7 +14175,7 @@
       <c r="F7" s="17"/>
     </row>
     <row r="8" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="32"/>
+      <c r="A8" s="30"/>
       <c r="B8" s="18">
         <v>2</v>
       </c>
@@ -14221,7 +14221,7 @@
       <c r="Z8" s="23"/>
     </row>
     <row r="9" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32"/>
+      <c r="A9" s="30"/>
       <c r="B9" s="18">
         <v>3</v>
       </c>
@@ -14251,7 +14251,7 @@
       <c r="Z9" s="23"/>
     </row>
     <row r="10" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="15"/>
       <c r="C10" s="16" t="s">
         <v>57</v>
@@ -14261,7 +14261,7 @@
       <c r="F10" s="17"/>
     </row>
     <row r="11" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="32"/>
+      <c r="A11" s="30"/>
       <c r="B11" s="24">
         <v>4</v>
       </c>
@@ -14291,7 +14291,7 @@
       </c>
     </row>
     <row r="12" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32"/>
+      <c r="A12" s="30"/>
       <c r="B12" s="24">
         <v>5</v>
       </c>
@@ -14305,7 +14305,7 @@
       <c r="F12" s="19"/>
     </row>
     <row r="13" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
+      <c r="A13" s="30"/>
       <c r="B13" s="18">
         <v>6</v>
       </c>
@@ -14319,7 +14319,7 @@
       <c r="F13" s="19"/>
     </row>
     <row r="14" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="32"/>
+      <c r="A14" s="30"/>
       <c r="B14" s="18">
         <v>7</v>
       </c>
@@ -14333,7 +14333,7 @@
       <c r="F14" s="19"/>
     </row>
     <row r="15" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32"/>
+      <c r="A15" s="30"/>
       <c r="B15" s="15"/>
       <c r="C15" s="16" t="s">
         <v>16</v>
@@ -14343,7 +14343,7 @@
       <c r="F15" s="17"/>
     </row>
     <row r="16" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="33"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="18">
         <v>7</v>
       </c>
@@ -14373,7 +14373,7 @@
       </c>
     </row>
     <row r="17" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="45" t="s">
+      <c r="A17" s="29" t="s">
         <v>82</v>
       </c>
       <c r="B17" s="15"/>
@@ -14385,7 +14385,7 @@
       <c r="F17" s="17"/>
     </row>
     <row r="18" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
+      <c r="A18" s="30"/>
       <c r="B18" s="18">
         <v>9</v>
       </c>
@@ -14415,7 +14415,7 @@
       </c>
     </row>
     <row r="19" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
+      <c r="A19" s="30"/>
       <c r="B19" s="24">
         <v>10</v>
       </c>
@@ -14429,7 +14429,7 @@
       <c r="F19" s="19"/>
     </row>
     <row r="20" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
+      <c r="A20" s="30"/>
       <c r="B20" s="18">
         <v>11</v>
       </c>
@@ -14463,7 +14463,7 @@
       <c r="Z20" s="23"/>
     </row>
     <row r="21" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="33"/>
+      <c r="A21" s="31"/>
       <c r="B21" s="18">
         <v>12</v>
       </c>
@@ -14477,7 +14477,7 @@
       <c r="F21" s="19"/>
     </row>
     <row r="22" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="45" t="s">
+      <c r="A22" s="29" t="s">
         <v>87</v>
       </c>
       <c r="B22" s="15"/>
@@ -14489,7 +14489,7 @@
       <c r="F22" s="17"/>
     </row>
     <row r="23" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32"/>
+      <c r="A23" s="30"/>
       <c r="B23" s="18">
         <v>17</v>
       </c>
@@ -14519,7 +14519,7 @@
       </c>
     </row>
     <row r="24" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="32"/>
+      <c r="A24" s="30"/>
       <c r="B24" s="18">
         <v>18</v>
       </c>
@@ -14533,7 +14533,7 @@
       <c r="F24" s="19"/>
     </row>
     <row r="25" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="32"/>
+      <c r="A25" s="30"/>
       <c r="B25" s="18">
         <v>19</v>
       </c>
@@ -14547,7 +14547,7 @@
       <c r="F25" s="19"/>
     </row>
     <row r="26" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="32"/>
+      <c r="A26" s="30"/>
       <c r="B26" s="18">
         <v>21</v>
       </c>
@@ -14561,7 +14561,7 @@
       <c r="F26" s="19"/>
     </row>
     <row r="27" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="33"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="18">
         <v>22</v>
       </c>
@@ -14575,7 +14575,7 @@
       <c r="F27" s="19"/>
     </row>
     <row r="28" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="45" t="s">
+      <c r="A28" s="29" t="s">
         <v>92</v>
       </c>
       <c r="B28" s="15"/>
@@ -14587,7 +14587,7 @@
       <c r="F28" s="17"/>
     </row>
     <row r="29" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="32"/>
+      <c r="A29" s="30"/>
       <c r="B29" s="18">
         <v>23</v>
       </c>
@@ -14617,7 +14617,7 @@
       </c>
     </row>
     <row r="30" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="32"/>
+      <c r="A30" s="30"/>
       <c r="B30" s="18">
         <v>24</v>
       </c>
@@ -14631,7 +14631,7 @@
       <c r="F30" s="19"/>
     </row>
     <row r="31" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="32"/>
+      <c r="A31" s="30"/>
       <c r="B31" s="18">
         <v>25</v>
       </c>
@@ -14645,7 +14645,7 @@
       <c r="F31" s="19"/>
     </row>
     <row r="32" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="32"/>
+      <c r="A32" s="30"/>
       <c r="B32" s="18">
         <v>26</v>
       </c>
@@ -14659,7 +14659,7 @@
       <c r="F32" s="19"/>
     </row>
     <row r="33" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32"/>
+      <c r="A33" s="30"/>
       <c r="B33" s="18">
         <v>27</v>
       </c>
@@ -14673,7 +14673,7 @@
       <c r="F33" s="19"/>
     </row>
     <row r="34" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="46"/>
+      <c r="A34" s="32"/>
       <c r="B34" s="18">
         <v>28</v>
       </c>
@@ -14687,7 +14687,7 @@
       <c r="F34" s="19"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="34" t="s">
+      <c r="A35" s="33" t="s">
         <v>69</v>
       </c>
       <c r="B35" s="15"/>
@@ -14699,7 +14699,7 @@
       <c r="F35" s="17"/>
     </row>
     <row r="36" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="35"/>
+      <c r="A36" s="34"/>
       <c r="B36" s="18">
         <v>29</v>
       </c>
@@ -14729,7 +14729,7 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="35"/>
+      <c r="A37" s="34"/>
       <c r="B37" s="18">
         <v>30</v>
       </c>
@@ -14743,7 +14743,7 @@
       <c r="F37" s="19"/>
     </row>
     <row r="38" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="35"/>
+      <c r="A38" s="34"/>
       <c r="B38" s="18">
         <v>31</v>
       </c>
@@ -14757,7 +14757,7 @@
       <c r="F38" s="19"/>
     </row>
     <row r="39" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="35"/>
+      <c r="A39" s="34"/>
       <c r="B39" s="15"/>
       <c r="C39" s="16" t="s">
         <v>25</v>
@@ -14767,7 +14767,7 @@
       <c r="F39" s="17"/>
     </row>
     <row r="40" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="35"/>
+      <c r="A40" s="34"/>
       <c r="B40" s="18">
         <v>32</v>
       </c>
@@ -14797,7 +14797,7 @@
       </c>
     </row>
     <row r="41" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="36"/>
+      <c r="A41" s="35"/>
       <c r="B41" s="18">
         <v>33</v>
       </c>
@@ -18689,37 +18689,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
     </row>
     <row r="2" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="30"/>
+      <c r="B2" s="38"/>
       <c r="C2" s="26"/>
       <c r="D2" s="40" t="s">
         <v>31</v>
       </c>
       <c r="E2" s="41"/>
-      <c r="F2" s="9" t="e">
+      <c r="F2" s="9">
         <f>COUNTIF(D5:D42,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="30"/>
+      <c r="B3" s="38"/>
       <c r="C3" s="10"/>
-      <c r="D3" s="47" t="s">
+      <c r="D3" s="42" t="s">
         <v>34</v>
       </c>
       <c r="E3" s="43"/>
@@ -18746,7 +18746,7 @@
       </c>
     </row>
     <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="29" t="s">
         <v>44</v>
       </c>
       <c r="B5" s="15"/>
@@ -18758,14 +18758,16 @@
       <c r="F5" s="17"/>
     </row>
     <row r="6" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="32"/>
+      <c r="A6" s="30"/>
       <c r="B6" s="18">
         <v>1</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="20"/>
+      <c r="D6" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="E6" s="19"/>
       <c r="F6" s="19"/>
       <c r="G6" s="5">
@@ -18782,11 +18784,11 @@
       </c>
       <c r="J6" s="5">
         <f>COUNTIF(D6,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="32"/>
+      <c r="A7" s="30"/>
       <c r="B7" s="15"/>
       <c r="C7" s="16" t="s">
         <v>14</v>
@@ -18795,20 +18797,22 @@
       <c r="E7" s="17"/>
       <c r="F7" s="17"/>
     </row>
-    <row r="8" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="32"/>
+    <row r="8" spans="1:26" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="30"/>
       <c r="B8" s="18">
         <v>2</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="20"/>
+      <c r="D8" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E8" s="19"/>
       <c r="F8" s="19"/>
       <c r="G8" s="5">
         <f>COUNTIF(D8,"Sim")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="5">
         <f>COUNTIF(D8,"Parcialmente")</f>
@@ -18840,7 +18844,7 @@
       <c r="Z8" s="23"/>
     </row>
     <row r="9" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32"/>
+      <c r="A9" s="30"/>
       <c r="B9" s="15"/>
       <c r="C9" s="16" t="s">
         <v>57</v>
@@ -18850,19 +18854,21 @@
       <c r="F9" s="17"/>
     </row>
     <row r="10" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="18">
         <v>3</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="D10" s="20"/>
+      <c r="D10" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E10" s="19"/>
       <c r="F10" s="19"/>
       <c r="G10" s="5">
         <f>COUNTIF(D10:D12,"Sim")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H10" s="5">
         <f>COUNTIF(D10:D12,"Parcialmente")</f>
@@ -18874,35 +18880,39 @@
       </c>
       <c r="J10" s="5">
         <f>COUNTIF(D10:D12,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="32"/>
+      <c r="A11" s="30"/>
       <c r="B11" s="18">
         <v>4</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="D11" s="20"/>
+      <c r="D11" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E11" s="19"/>
       <c r="F11" s="19"/>
     </row>
     <row r="12" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32"/>
+      <c r="A12" s="30"/>
       <c r="B12" s="18">
         <v>5</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="D12" s="20"/>
+      <c r="D12" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="E12" s="19"/>
       <c r="F12" s="19"/>
     </row>
     <row r="13" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
+      <c r="A13" s="30"/>
       <c r="B13" s="15"/>
       <c r="C13" s="16" t="s">
         <v>16</v>
@@ -18912,14 +18922,16 @@
       <c r="F13" s="17"/>
     </row>
     <row r="14" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="33"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="18">
         <v>6</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="20"/>
+      <c r="D14" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="E14" s="19"/>
       <c r="F14" s="19"/>
       <c r="G14" s="5">
@@ -18936,11 +18948,11 @@
       </c>
       <c r="J14" s="5">
         <f>COUNTIF(D14,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="45" t="s">
+      <c r="A15" s="29" t="s">
         <v>82</v>
       </c>
       <c r="B15" s="15"/>
@@ -18952,14 +18964,16 @@
       <c r="F15" s="17"/>
     </row>
     <row r="16" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="33"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="18">
         <v>8</v>
       </c>
       <c r="C16" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="D16" s="20"/>
+      <c r="D16" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="E16" s="19"/>
       <c r="F16" s="19"/>
       <c r="G16" s="5">
@@ -18976,11 +18990,11 @@
       </c>
       <c r="J16" s="5">
         <f>COUNTIF(D16,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="45" t="s">
+      <c r="A17" s="29" t="s">
         <v>87</v>
       </c>
       <c r="B17" s="15"/>
@@ -18992,19 +19006,21 @@
       <c r="F17" s="17"/>
     </row>
     <row r="18" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
+      <c r="A18" s="30"/>
       <c r="B18" s="18">
         <v>11</v>
       </c>
       <c r="C18" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="D18" s="20"/>
+      <c r="D18" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E18" s="19"/>
       <c r="F18" s="19"/>
       <c r="G18" s="5">
         <f>COUNTIF(D18:D22,"Sim")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18" s="5">
         <f>COUNTIF(D18:D22,"Parcialmente")</f>
@@ -19012,7 +19028,7 @@
       </c>
       <c r="I18" s="5">
         <f>COUNTIF(D18:D22,"Não")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" s="5">
         <f>COUNTIF(D18:D22,"NA")</f>
@@ -19020,55 +19036,63 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
+      <c r="A19" s="30"/>
       <c r="B19" s="18">
         <v>13</v>
       </c>
       <c r="C19" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="D19" s="20"/>
+      <c r="D19" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E19" s="19"/>
       <c r="F19" s="19"/>
     </row>
     <row r="20" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
+      <c r="A20" s="30"/>
       <c r="B20" s="18">
         <v>14</v>
       </c>
       <c r="C20" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="20"/>
+      <c r="D20" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E20" s="19"/>
       <c r="F20" s="19"/>
     </row>
     <row r="21" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="32"/>
+      <c r="A21" s="30"/>
       <c r="B21" s="18">
         <v>15</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="20"/>
+      <c r="D21" s="20" t="s">
+        <v>43</v>
+      </c>
       <c r="E21" s="19"/>
       <c r="F21" s="19"/>
     </row>
     <row r="22" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="33"/>
+      <c r="A22" s="31"/>
       <c r="B22" s="18">
         <v>16</v>
       </c>
       <c r="C22" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="D22" s="20"/>
+      <c r="D22" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E22" s="19"/>
       <c r="F22" s="19"/>
     </row>
     <row r="23" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="45" t="s">
+      <c r="A23" s="29" t="s">
         <v>104</v>
       </c>
       <c r="B23" s="15"/>
@@ -19080,19 +19104,21 @@
       <c r="F23" s="17"/>
     </row>
     <row r="24" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="32"/>
+      <c r="A24" s="30"/>
       <c r="B24" s="24">
         <v>17</v>
       </c>
       <c r="C24" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="D24" s="20"/>
+      <c r="D24" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E24" s="19"/>
       <c r="F24" s="19"/>
       <c r="G24" s="5">
         <f>COUNTIF(D24:D28,"Sim")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H24" s="5">
         <f>COUNTIF(D24:D28,"Parcialmente")</f>
@@ -19104,59 +19130,67 @@
       </c>
       <c r="J24" s="5">
         <f>COUNTIF(D24:D28,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="32"/>
+      <c r="A25" s="30"/>
       <c r="B25" s="18">
         <v>18</v>
       </c>
       <c r="C25" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D25" s="20"/>
+      <c r="D25" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E25" s="19"/>
       <c r="F25" s="19"/>
     </row>
     <row r="26" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="32"/>
+      <c r="A26" s="30"/>
       <c r="B26" s="18">
         <v>19</v>
       </c>
       <c r="C26" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D26" s="20"/>
+      <c r="D26" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E26" s="19"/>
       <c r="F26" s="19"/>
     </row>
     <row r="27" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="32"/>
+      <c r="A27" s="30"/>
       <c r="B27" s="18">
         <v>21</v>
       </c>
       <c r="C27" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D27" s="20"/>
+      <c r="D27" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="E27" s="19"/>
       <c r="F27" s="19"/>
     </row>
     <row r="28" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="33"/>
+      <c r="A28" s="31"/>
       <c r="B28" s="18">
         <v>22</v>
       </c>
       <c r="C28" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="D28" s="20"/>
+      <c r="D28" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E28" s="19"/>
       <c r="F28" s="19"/>
     </row>
     <row r="29" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="29" t="s">
         <v>92</v>
       </c>
       <c r="B29" s="15"/>
@@ -19168,19 +19202,21 @@
       <c r="F29" s="17"/>
     </row>
     <row r="30" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="32"/>
+      <c r="A30" s="30"/>
       <c r="B30" s="18">
         <v>24</v>
       </c>
       <c r="C30" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="D30" s="20"/>
+      <c r="D30" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E30" s="19"/>
       <c r="F30" s="19"/>
       <c r="G30" s="5">
         <f>COUNTIF(D30:D34,"Sim")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H30" s="5">
         <f>COUNTIF(D30:D34,"Parcialmente")</f>
@@ -19192,59 +19228,67 @@
       </c>
       <c r="J30" s="5">
         <f>COUNTIF(D30:D34,"NA")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="32"/>
+      <c r="A31" s="30"/>
       <c r="B31" s="18">
         <v>26</v>
       </c>
       <c r="C31" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="D31" s="20"/>
+      <c r="D31" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="E31" s="19"/>
       <c r="F31" s="19"/>
     </row>
     <row r="32" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="32"/>
+      <c r="A32" s="30"/>
       <c r="B32" s="18">
         <v>27</v>
       </c>
       <c r="C32" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="D32" s="20"/>
+      <c r="D32" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E32" s="19"/>
       <c r="F32" s="19"/>
     </row>
     <row r="33" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32"/>
+      <c r="A33" s="30"/>
       <c r="B33" s="18">
         <v>28</v>
       </c>
       <c r="C33" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="D33" s="20"/>
+      <c r="D33" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="E33" s="19"/>
       <c r="F33" s="19"/>
     </row>
     <row r="34" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="46"/>
+      <c r="A34" s="32"/>
       <c r="B34" s="18">
         <v>29</v>
       </c>
       <c r="C34" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="D34" s="20"/>
+      <c r="D34" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="E34" s="19"/>
       <c r="F34" s="19"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="34" t="s">
+      <c r="A35" s="33" t="s">
         <v>69</v>
       </c>
       <c r="B35" s="15"/>
@@ -19256,19 +19300,21 @@
       <c r="F35" s="17"/>
     </row>
     <row r="36" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="35"/>
+      <c r="A36" s="34"/>
       <c r="B36" s="18">
         <v>30</v>
       </c>
       <c r="C36" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="D36" s="20"/>
+      <c r="D36" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E36" s="19"/>
       <c r="F36" s="19"/>
       <c r="G36" s="5">
         <f>COUNTIF(D36:D38,"Sim")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H36" s="5">
         <f>COUNTIF(D36:D38,"Parcialmente")</f>
@@ -19284,41 +19330,47 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="35"/>
+      <c r="A37" s="34"/>
       <c r="B37" s="18">
         <v>31</v>
       </c>
       <c r="C37" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="D37" s="20"/>
+      <c r="D37" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E37" s="19"/>
       <c r="F37" s="19"/>
     </row>
     <row r="38" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="35"/>
+      <c r="A38" s="34"/>
       <c r="B38" s="18">
         <v>32</v>
       </c>
       <c r="C38" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="D38" s="20"/>
+      <c r="D38" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E38" s="19"/>
       <c r="F38" s="19"/>
     </row>
     <row r="39" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="35"/>
+      <c r="A39" s="34"/>
       <c r="B39" s="18"/>
       <c r="C39" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="D39" s="20"/>
+      <c r="D39" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E39" s="19"/>
       <c r="F39" s="19"/>
     </row>
     <row r="40" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="35"/>
+      <c r="A40" s="34"/>
       <c r="B40" s="15"/>
       <c r="C40" s="16" t="s">
         <v>25</v>
@@ -19328,19 +19380,21 @@
       <c r="F40" s="17"/>
     </row>
     <row r="41" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="35"/>
+      <c r="A41" s="34"/>
       <c r="B41" s="18">
         <v>33</v>
       </c>
       <c r="C41" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D41" s="20"/>
+      <c r="D41" s="20" t="s">
+        <v>55</v>
+      </c>
       <c r="E41" s="19"/>
       <c r="F41" s="19"/>
       <c r="G41" s="5">
         <f>COUNTIF(D41:D42,"Sim")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H41" s="5">
         <f>COUNTIF(D41:D42,"Parcialmente")</f>
@@ -19352,18 +19406,20 @@
       </c>
       <c r="J41" s="5">
         <f>COUNTIF(D41:D42,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="36"/>
+      <c r="A42" s="35"/>
       <c r="B42" s="18">
         <v>34</v>
       </c>
       <c r="C42" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="D42" s="20"/>
+      <c r="D42" s="20" t="s">
+        <v>46</v>
+      </c>
       <c r="E42" s="19"/>
       <c r="F42" s="19"/>
     </row>
@@ -23222,20 +23278,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
     </row>
     <row r="2" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="30"/>
+      <c r="B2" s="38"/>
       <c r="C2" s="26"/>
       <c r="D2" s="40" t="s">
         <v>31</v>
@@ -23250,9 +23306,9 @@
       <c r="A3" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="30"/>
+      <c r="B3" s="38"/>
       <c r="C3" s="10"/>
-      <c r="D3" s="47" t="s">
+      <c r="D3" s="42" t="s">
         <v>34</v>
       </c>
       <c r="E3" s="43"/>
@@ -23279,7 +23335,7 @@
       </c>
     </row>
     <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="29" t="s">
         <v>44</v>
       </c>
       <c r="B5" s="15"/>
@@ -23291,7 +23347,7 @@
       <c r="F5" s="17"/>
     </row>
     <row r="6" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="32"/>
+      <c r="A6" s="30"/>
       <c r="B6" s="18">
         <v>1</v>
       </c>
@@ -23319,7 +23375,7 @@
       </c>
     </row>
     <row r="7" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="32"/>
+      <c r="A7" s="30"/>
       <c r="B7" s="15"/>
       <c r="C7" s="16" t="s">
         <v>14</v>
@@ -23329,7 +23385,7 @@
       <c r="F7" s="17"/>
     </row>
     <row r="8" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="32"/>
+      <c r="A8" s="30"/>
       <c r="B8" s="18">
         <v>2</v>
       </c>
@@ -23373,7 +23429,7 @@
       <c r="Z8" s="23"/>
     </row>
     <row r="9" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32"/>
+      <c r="A9" s="30"/>
       <c r="B9" s="15"/>
       <c r="C9" s="16" t="s">
         <v>15</v>
@@ -23383,7 +23439,7 @@
       <c r="F9" s="17"/>
     </row>
     <row r="10" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="18">
         <v>3</v>
       </c>
@@ -23411,7 +23467,7 @@
       </c>
     </row>
     <row r="11" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="32"/>
+      <c r="A11" s="30"/>
       <c r="B11" s="18">
         <v>4</v>
       </c>
@@ -23423,7 +23479,7 @@
       <c r="F11" s="19"/>
     </row>
     <row r="12" spans="1:26" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32"/>
+      <c r="A12" s="30"/>
       <c r="B12" s="18">
         <v>5</v>
       </c>
@@ -23435,7 +23491,7 @@
       <c r="F12" s="19"/>
     </row>
     <row r="13" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
+      <c r="A13" s="30"/>
       <c r="B13" s="15"/>
       <c r="C13" s="16" t="s">
         <v>16</v>
@@ -23445,7 +23501,7 @@
       <c r="F13" s="17"/>
     </row>
     <row r="14" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="33"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="18">
         <v>6</v>
       </c>
@@ -23473,7 +23529,7 @@
       </c>
     </row>
     <row r="15" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="45" t="s">
+      <c r="A15" s="29" t="s">
         <v>82</v>
       </c>
       <c r="B15" s="15"/>
@@ -23485,7 +23541,7 @@
       <c r="F15" s="17"/>
     </row>
     <row r="16" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="33"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="18">
         <v>8</v>
       </c>
@@ -23513,7 +23569,7 @@
       </c>
     </row>
     <row r="17" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="45" t="s">
+      <c r="A17" s="29" t="s">
         <v>87</v>
       </c>
       <c r="B17" s="15"/>
@@ -23525,7 +23581,7 @@
       <c r="F17" s="17"/>
     </row>
     <row r="18" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
+      <c r="A18" s="30"/>
       <c r="B18" s="18">
         <v>9</v>
       </c>
@@ -23553,7 +23609,7 @@
       </c>
     </row>
     <row r="19" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
+      <c r="A19" s="30"/>
       <c r="B19" s="18">
         <v>10</v>
       </c>
@@ -23565,7 +23621,7 @@
       <c r="F19" s="19"/>
     </row>
     <row r="20" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
+      <c r="A20" s="30"/>
       <c r="B20" s="18">
         <v>11</v>
       </c>
@@ -23577,7 +23633,7 @@
       <c r="F20" s="19"/>
     </row>
     <row r="21" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="46"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="18">
         <v>13</v>
       </c>
@@ -23589,7 +23645,7 @@
       <c r="F21" s="19"/>
     </row>
     <row r="22" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="45" t="s">
+      <c r="A22" s="29" t="s">
         <v>104</v>
       </c>
       <c r="B22" s="15"/>
@@ -23601,7 +23657,7 @@
       <c r="F22" s="17"/>
     </row>
     <row r="23" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32"/>
+      <c r="A23" s="30"/>
       <c r="B23" s="18">
         <v>14</v>
       </c>
@@ -23629,7 +23685,7 @@
       </c>
     </row>
     <row r="24" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="33"/>
+      <c r="A24" s="31"/>
       <c r="B24" s="18">
         <v>15</v>
       </c>
@@ -23641,7 +23697,7 @@
       <c r="F24" s="19"/>
     </row>
     <row r="25" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="45" t="s">
+      <c r="A25" s="29" t="s">
         <v>116</v>
       </c>
       <c r="B25" s="15"/>
@@ -23673,7 +23729,7 @@
       <c r="Z25" s="23"/>
     </row>
     <row r="26" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="32"/>
+      <c r="A26" s="30"/>
       <c r="B26" s="24">
         <v>24</v>
       </c>
@@ -23717,7 +23773,7 @@
       <c r="Z26" s="23"/>
     </row>
     <row r="27" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="32"/>
+      <c r="A27" s="30"/>
       <c r="B27" s="18">
         <v>25</v>
       </c>
@@ -23749,7 +23805,7 @@
       <c r="Z27" s="23"/>
     </row>
     <row r="28" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="32"/>
+      <c r="A28" s="30"/>
       <c r="B28" s="15"/>
       <c r="C28" s="16" t="s">
         <v>28</v>
@@ -23759,7 +23815,7 @@
       <c r="F28" s="17"/>
     </row>
     <row r="29" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="33"/>
+      <c r="A29" s="31"/>
       <c r="B29" s="24">
         <v>26</v>
       </c>
@@ -23787,7 +23843,7 @@
       </c>
     </row>
     <row r="30" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="29" t="s">
         <v>92</v>
       </c>
       <c r="B30" s="15"/>
@@ -23799,7 +23855,7 @@
       <c r="F30" s="17"/>
     </row>
     <row r="31" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="32"/>
+      <c r="A31" s="30"/>
       <c r="B31" s="18">
         <v>19</v>
       </c>
@@ -23827,7 +23883,7 @@
       </c>
     </row>
     <row r="32" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="32"/>
+      <c r="A32" s="30"/>
       <c r="B32" s="18">
         <v>20</v>
       </c>
@@ -23839,7 +23895,7 @@
       <c r="F32" s="19"/>
     </row>
     <row r="33" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32"/>
+      <c r="A33" s="30"/>
       <c r="B33" s="18">
         <v>21</v>
       </c>
@@ -23851,7 +23907,7 @@
       <c r="F33" s="19"/>
     </row>
     <row r="34" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="32"/>
+      <c r="A34" s="30"/>
       <c r="B34" s="18">
         <v>24</v>
       </c>
@@ -23863,7 +23919,7 @@
       <c r="F34" s="19"/>
     </row>
     <row r="35" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="46"/>
+      <c r="A35" s="32"/>
       <c r="B35" s="18">
         <v>25</v>
       </c>
@@ -23875,7 +23931,7 @@
       <c r="F35" s="19"/>
     </row>
     <row r="36" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="34" t="s">
+      <c r="A36" s="33" t="s">
         <v>69</v>
       </c>
       <c r="B36" s="15"/>
@@ -23887,7 +23943,7 @@
       <c r="F36" s="17"/>
     </row>
     <row r="37" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="35"/>
+      <c r="A37" s="34"/>
       <c r="B37" s="18">
         <v>26</v>
       </c>
@@ -23915,7 +23971,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="35"/>
+      <c r="A38" s="34"/>
       <c r="B38" s="18">
         <v>27</v>
       </c>
@@ -23927,7 +23983,7 @@
       <c r="F38" s="19"/>
     </row>
     <row r="39" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="35"/>
+      <c r="A39" s="34"/>
       <c r="B39" s="18">
         <v>28</v>
       </c>
@@ -23939,7 +23995,7 @@
       <c r="F39" s="19"/>
     </row>
     <row r="40" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="35"/>
+      <c r="A40" s="34"/>
       <c r="B40" s="18"/>
       <c r="C40" s="19" t="s">
         <v>111</v>
@@ -23949,7 +24005,7 @@
       <c r="F40" s="19"/>
     </row>
     <row r="41" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="35"/>
+      <c r="A41" s="34"/>
       <c r="B41" s="15"/>
       <c r="C41" s="16" t="s">
         <v>25</v>
@@ -23959,7 +24015,7 @@
       <c r="F41" s="17"/>
     </row>
     <row r="42" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="35"/>
+      <c r="A42" s="34"/>
       <c r="B42" s="18">
         <v>29</v>
       </c>
@@ -23987,7 +24043,7 @@
       </c>
     </row>
     <row r="43" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="36"/>
+      <c r="A43" s="35"/>
       <c r="B43" s="18">
         <v>30</v>
       </c>
@@ -27807,6 +27863,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A25:A29"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="A36:A43"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A1:F1"/>
@@ -27814,11 +27875,6 @@
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="D3:F3"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="A25:A29"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="A36:A43"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D15 D17 D22 D25 D28 D30 D36 D41" xr:uid="{00000000-0002-0000-0500-000000000000}">

</xml_diff>